<commit_message>
eval(assistant): business vocabulary experiment
Adds four real questions about employee onboarding and invoice cancellation to question set v2, including the same question with and without an initial capital letter. calibrate_vocab.py boosts chunks of the topics detected from the question with a seed vocabulary, an automatic one (distinctive words of each topic's manuals) or both, at several strengths, with and without query normalization, on top of the production configuration. Saves a draft vocabulary for review. Production is unchanged.
</commit_message>
<xml_diff>
--- a/backend/assistant-service/evaluation/datasets/preguntas-v2.xlsx
+++ b/backend/assistant-service/evaluation/datasets/preguntas-v2.xlsx
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="11" min="1" max="1"/>
@@ -1602,165 +1602,297 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>P26</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>¿Cómo veo mi stock?</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>totvs-stock-costos</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-stock-costos-v2.pdf</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="11" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="G28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>P27</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>¿Dónde consulto un producto de stock?</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>ubicacion</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>totvs-stock-costos</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>capacitacion-2026-09-08.transcripcion.docx</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>22:03</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>P28</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>¿Cómo calculo la nómina?</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>totvs-nomina</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-nomina-v2.pdf</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="11" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="G30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>P29</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>¿Cómo timbro una factura en TOTVS?</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="11" t="inlineStr">
         <is>
           <t>totvs-ventas-facturacion</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-ventas-facturacion-v2.pdf</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="11" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" s="11" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>P30</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>¿Por qué me marca error al borrar una factura?</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>ninguno</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="F32" s="11" t="inlineStr"/>
+      <c r="G32" s="11" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>P31</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Como doy de alta un empleado?</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>proceso</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>totvs-nomina</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>manual-autocapacitacion-nomina-v2.pdf</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>P32</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>como doy de alta un empleado?</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>proceso</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>totvs-nomina</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>manual-autocapacitacion-nomina-v2.pdf</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>P33</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>como creo un empleado en nomina?</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>proceso</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>totvs-nomina</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>manual-autocapacitacion-nomina-v2.pdf</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>P34</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Porque no puedo cancelar una Factura?</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>proceso</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>totvs-ventas-facturacion</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>manual-autocapacitacion-ventas-facturacion-v2.pdf</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>

<commit_message>
eval(assistant): Spanish stemming experiment for BM25
Adds a real user question (P35, 'no se como facturar una venta') whose answer ranked fifth with low confidence because BM25 compared 'facturar' with 'factura' as different words. calibrate_stem.py compares the current BM25 with a Snowball Spanish stemmed BM25 on the production configuration. Production is unchanged.
</commit_message>
<xml_diff>
--- a/backend/assistant-service/evaluation/datasets/preguntas-v2.xlsx
+++ b/backend/assistant-service/evaluation/datasets/preguntas-v2.xlsx
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="11" min="1" max="1"/>
@@ -1763,136 +1763,169 @@
       <c r="G32" s="11" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>P31</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>Como doy de alta un empleado?</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="11" t="inlineStr">
         <is>
           <t>totvs-nomina</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-nomina-v2.pdf</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="11" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>P32</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>como doy de alta un empleado?</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
         <is>
           <t>totvs-nomina</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-nomina-v2.pdf</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="11" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="G34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>P33</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>como creo un empleado en nomina?</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="11" t="inlineStr">
         <is>
           <t>totvs-nomina</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-nomina-v2.pdf</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="G35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>P34</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Porque no puedo cancelar una Factura?</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>proceso</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>totvs-ventas-facturacion</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>manual-autocapacitacion-ventas-facturacion-v2.pdf</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="11" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="G36" s="11" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>P35</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>no se como facturar una venta</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>proceso</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>totvs-ventas-facturacion</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>manual-autocapacitacion-ventas-facturacion-v2.pdf</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">

</xml_diff>